<commit_message>
fix: harden workbook and report deliverables
</commit_message>
<xml_diff>
--- a/deliverables/Setup-Sahla-Launch-Workbook.xlsx
+++ b/deliverables/Setup-Sahla-Launch-Workbook.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Dashboard" sheetId="1" r:id="R5da13c24a2ef444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R2648346d5fa14757"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Providers" sheetId="3" r:id="Ra486513141a24c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R5204230d643b40cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="5" r:id="Reb68ba3c70f348cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Map" sheetId="6" r:id="Rdb42fe0e16a34581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Actions" sheetId="7" r:id="Rba2c03a7f8c14aa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Dashboard" sheetId="1" r:id="R7f73336ef7d94791"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="2" r:id="R172274209a03457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Providers" sheetId="3" r:id="R2fd2578856444878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keywords" sheetId="4" r:id="R315ab0df456d4fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="5" r:id="R4c84c816b1824069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Map" sheetId="6" r:id="R96e55385bd5c4d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner Actions" sheetId="7" r:id="R89f4a2d9071046b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,8 +16,8 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={7402CA00-0C59-7E9F-4284-84B6E9CD997C}</x:author>
-    <x:author>tc={AB6BADF6-FA37-FC64-9E8D-BD55B83D6F40}</x:author>
+    <x:author>tc={505D1BEA-0B1E-141A-96B1-04C9D02546EF}</x:author>
+    <x:author>tc={20A62CC2-7BD1-4C27-5650-4F1C2B50451F}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="A10" authorId="0">
@@ -36,7 +36,7 @@
           <x:t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Formula-backed average of the five visible product totals. Each product total is the sum of seven visible selection components; the score is an editorial rank inside the evaluated launch set, not a performance claim.</x:t>
+    Formula-backed average of the five visible product totals. Each product total is the sum of seven visible selection components; the score ranks evidence-qualified launch products inside the evaluated candidate set. It is not a performance score or trend validation.</x:t>
         </x:r>
       </x:text>
     </x:comment>
@@ -719,7 +719,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>Launch selection score / 100</a:t>
+              <a:t>Evidence-qualified launch selection score / 100</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -856,7 +856,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra5e5e634a6754a58"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra33b5f7e33e04c16"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -877,13 +877,13 @@
     <xdr:ext cx="1066800" cy="685800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="1a6eccdb-5c3c-403d-a53a-9b87285fd94b"/>
+        <xdr:cNvPr id="1" name="63a5276f-4391-48a1-9ae7-b4a00abcc6b4"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5aeceb0ca0794f7d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R93220c32599c4c6c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -904,13 +904,13 @@
     <xdr:ext cx="1066800" cy="685800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="97798d2a-a47c-4039-922b-9a054136b12d"/>
+        <xdr:cNvPr id="2" name="3faa31b2-d406-4ee3-b9c2-aa96de20f0c4"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3b1cac9d15554d8c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3a7425e078514dc0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -931,13 +931,13 @@
     <xdr:ext cx="1066800" cy="685800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="7721d502-4319-4a73-b37e-dc00c03ecd7b"/>
+        <xdr:cNvPr id="3" name="c0ca00a2-4a64-4231-a3d5-2a2016b37ba0"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1ec93e8b5cca4018"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf4ddaed2d8164af1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -958,13 +958,13 @@
     <xdr:ext cx="1066800" cy="685800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="767e8827-c4d2-481e-81da-328cb2d45f2a"/>
+        <xdr:cNvPr id="4" name="35a0a49e-64c3-430d-ae4d-2cc6ed959ba9"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0133dbaad1554f83"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raea7d0a0088746c6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -985,13 +985,13 @@
     <xdr:ext cx="1066800" cy="685800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="e4a3e969-1b5a-47e5-8c87-89a7813326a5"/>
+        <xdr:cNvPr id="5" name="bc959b8b-4d05-4d65-9766-19d484fd934d"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcbb1a223cf5e4dda"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5166b544c9384369"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1007,7 +1007,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="Setup Sahla" id="{F9A69630-CBA1-4341-B873-028EAB4E98EF}"/>
+  <xltc:person displayName="Setup Sahla" id="{AB6F446B-B398-4B00-8563-9B63C79A1928}"/>
 </xltc:personList>
 </file>
 
@@ -1336,17 +1336,17 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="A10" dT="2026-07-15T01:46:10.837" personId="{F9A69630-CBA1-4341-B873-028EAB4E98EF}" id="{7402CA00-0C59-7E9F-4284-84B6E9CD997C}">
+  <xltc:threadedComment ref="A10" dT="2026-07-15T02:21:58.017" personId="{AB6F446B-B398-4B00-8563-9B63C79A1928}" id="{505D1BEA-0B1E-141A-96B1-04C9D02546EF}">
     <xltc:text>Source: docs/business/AFFILIATE_ACTIVATION.md and research/affiliate-program-evidence.csv. Affiliate IDs and Noon Egypt territory permission are owner-controlled inputs and are not present in this launch package.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="J5" dT="2026-07-15T01:46:10.838" personId="{F9A69630-CBA1-4341-B873-028EAB4E98EF}" id="{AB6BADF6-FA37-FC64-9E8D-BD55B83D6F40}">
-    <xltc:text>Formula-backed average of the five visible product totals. Each product total is the sum of seven visible selection components; the score is an editorial rank inside the evaluated launch set, not a performance claim.</xltc:text>
+  <xltc:threadedComment ref="J5" dT="2026-07-15T02:21:58.017" personId="{AB6F446B-B398-4B00-8563-9B63C79A1928}" id="{20A62CC2-7BD1-4C27-5650-4F1C2B50451F}">
+    <xltc:text>Formula-backed average of the five visible product totals. Each product total is the sum of seven visible selection components; the score ranks evidence-qualified launch products inside the evaluated candidate set. It is not a performance score or trend validation.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
@@ -1419,52 +1419,52 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="L2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="M2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="N2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="O2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
       <x:c r="P2" s="7" t="str">
-        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
+        <x:v>Fix the friction. Keep the gear. Egypt-first launch package with five evidence-qualified product routes, three guides, dated provider evidence, original visuals, and direct links pending owner affiliate activation.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="9" customHeight="1"/>
@@ -1854,7 +1854,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B16" s="124" t="str">
-        <x:v>Autocomplete presence is qualitative search-language evidence, not search volume or trend strength.</x:v>
+        <x:v>No volume/trend-direction/growth dataset was available. These are evidence-qualified launch products, not trend-validated winners.</x:v>
       </x:c>
       <x:c r="C16" s="124"/>
       <x:c r="D16" s="124"/>
@@ -2071,13 +2071,13 @@
     <x:mergeCell ref="C29:D29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf38862490eb4b3f"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R104ed6d5c3424b54"/>
+  <x:drawing r:id="R7b4e520e303a495f"/>
+  <x:legacyDrawing r:id="Rd55fb0d548a74b44"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns3="http://schemas.microsoft.com/office/excel/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
@@ -2104,126 +2104,126 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="C1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="D1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="G1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="H1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="I1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="J1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="K1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="L1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="M1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="N1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="O1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="P1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="Q1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="R1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="S1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
       <x:c r="T1" s="3" t="str">
-        <x:v>SETUP SAHLA / SELECTED PRODUCTS</x:v>
+        <x:v>SETUP SAHLA / EVIDENCE-QUALIFIED PRODUCTS</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="L2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="M2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="N2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="O2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="P2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="Q2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="R2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="S2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
       <x:c r="T2" s="7" t="str">
-        <x:v>Five launch products. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
+        <x:v>Five evidence-qualified launch products, not trend-validated winners. Total score is formula-driven from seven visible components. Prices are dated EGP snapshots, not current-price claims.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="9" customHeight="1"/>
@@ -2617,38 +2617,38 @@
         <x:color rgb="FFC9FF4A"/>
       </x:dataBar>
       <x:extLst>
-        <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{ED752712-34E2-97EC-30C1-25647B402030}</x14:id>
+        <x:ext uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <ns1:id>{ED752712-34E2-97EC-30C1-25647B402030}</ns1:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdaa1343b90fc4ab6"/>
+  <x:drawing r:id="R65ed966978704699"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ec73ea5d014ceb"/>
+    <x:tablePart r:id="R650107c9f0a14d09"/>
   </x:tableParts>
   <x:extLst>
-    <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting>
-          <x14:cfRule type="dataBar" priority="1" id="{ED752712-34E2-97EC-30C1-25647B402030}">
-            <x14:dataBar gradient="0">
-              <x14:cfvo type="min"/>
-              <x14:cfvo type="max"/>
-              <x14:fillColor rgb="FFC9FF4A"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>K6:K10</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
+    <x:ext uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <ns1:conditionalFormattings>
+        <ns1:conditionalFormatting>
+          <ns1:cfRule type="dataBar" priority="1" id="{ED752712-34E2-97EC-30C1-25647B402030}">
+            <ns1:dataBar gradient="0">
+              <ns1:cfvo type="min"/>
+              <ns1:cfvo type="max"/>
+              <ns1:fillColor rgb="FFC9FF4A"/>
+            </ns1:dataBar>
+          </ns1:cfRule>
+          <ns3:sqref>K6:K10</ns3:sqref>
+        </ns1:conditionalFormatting>
+      </ns1:conditionalFormattings>
     </x:ext>
   </x:extLst>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
@@ -2805,16 +2805,14 @@
       <x:c r="H6" s="25" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="I6" s="40" t="e">
-        <x:f>HYPERLINK("https://www.amazon.eg/-/en/dp/B0BQLLB61B","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.amazon.eg/-/en/dp/B0BQLLB61B, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I6" s="40" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J6" s="25" t="str">
         <x:v>https://www.amazon.eg/-/en/dp/B0BQLLB61B</x:v>
       </x:c>
-      <x:c r="K6" s="40" t="e">
-        <x:f>HYPERLINK("https://www.anker.com/products/a8355","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.anker.com/products/a8355, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K6" s="40" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
         <x:v>https://www.anker.com/products/a8355</x:v>
@@ -2845,16 +2843,14 @@
       <x:c r="H7" s="26" t="str">
         <x:v>Unverified — public terms do not establish Egypt eligibility</x:v>
       </x:c>
-      <x:c r="I7" s="41" t="e">
-        <x:f>HYPERLINK("https://www.noon.com/egypt-en/anker-332-usb-c-hub-5-in-1-usb-c-connector-with-4k-hdmi-100w-power-charger-black-a8355h11/N70086896V/p/","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.noon.com/egypt-en/anker-332-usb-c-hub-5-in-1-usb-c-connector-with-4k-hdmi-100w-power-charger-black-a8355h11/N70086896V/p/, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I7" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J7" s="26" t="str">
         <x:v>https://www.noon.com/egypt-en/anker-332-usb-c-hub-5-in-1-usb-c-connector-with-4k-hdmi-100w-power-charger-black-a8355h11/N70086896V/p/</x:v>
       </x:c>
-      <x:c r="K7" s="41" t="e">
-        <x:f>HYPERLINK("https://www.anker.com/products/a8355","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.anker.com/products/a8355, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K7" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L7" s="26" t="str">
         <x:v>https://www.anker.com/products/a8355</x:v>
@@ -2885,16 +2881,14 @@
       <x:c r="H8" s="26" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="I8" s="41" t="e">
-        <x:f>HYPERLINK("https://www.amazon.eg/-/en/dp/B08TLVKBMJ","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.amazon.eg/-/en/dp/B08TLVKBMJ, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I8" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J8" s="26" t="str">
         <x:v>https://www.amazon.eg/-/en/dp/B08TLVKBMJ</x:v>
       </x:c>
-      <x:c r="K8" s="41" t="e">
-        <x:f>HYPERLINK("https://www.ugreen.com/tr-tr/products/tr-40289","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.ugreen.com/tr-tr/products/tr-40289, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K8" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L8" s="26" t="str">
         <x:v>https://www.ugreen.com/tr-tr/products/tr-40289</x:v>
@@ -2925,16 +2919,14 @@
       <x:c r="H9" s="26" t="str">
         <x:v>Unverified — public terms do not establish Egypt eligibility</x:v>
       </x:c>
-      <x:c r="I9" s="41" t="e">
-        <x:f>HYPERLINK("https://www.noon.com/egypt-en/laptop-stand-aluminum-alloy-adjustable-eye-level-ergonomic-height-laptop-riser-holder-compatible-for-macbook-pro-2021-air-chromebook-and-more-storage-bag-included/N53340883A/p/","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.noon.com/egypt-en/laptop-stand-aluminum-alloy-adjustable-eye-level-ergonomic-height-laptop-riser-holder-compatible-for-macbook-pro-2021-air-chromebook-and-more-storage-bag-included/N53340883A/p/, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I9" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J9" s="26" t="str">
         <x:v>https://www.noon.com/egypt-en/laptop-stand-aluminum-alloy-adjustable-eye-level-ergonomic-height-laptop-riser-holder-compatible-for-macbook-pro-2021-air-chromebook-and-more-storage-bag-included/N53340883A/p/</x:v>
       </x:c>
-      <x:c r="K9" s="41" t="e">
-        <x:f>HYPERLINK("https://www.ugreen.com/tr-tr/products/tr-40289","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.ugreen.com/tr-tr/products/tr-40289, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K9" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L9" s="26" t="str">
         <x:v>https://www.ugreen.com/tr-tr/products/tr-40289</x:v>
@@ -2965,16 +2957,14 @@
       <x:c r="H10" s="26" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="I10" s="41" t="e">
-        <x:f>HYPERLINK("https://www.amazon.eg/-/en/dp/B0CP198X1G","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.amazon.eg/-/en/dp/B0CP198X1G, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I10" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J10" s="26" t="str">
         <x:v>https://www.amazon.eg/-/en/dp/B0CP198X1G</x:v>
       </x:c>
-      <x:c r="K10" s="41" t="e">
-        <x:f>HYPERLINK("https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K10" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L10" s="26" t="str">
         <x:v>https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop</x:v>
@@ -3005,16 +2995,14 @@
       <x:c r="H11" s="26" t="str">
         <x:v>Unverified — public terms do not establish Egypt eligibility</x:v>
       </x:c>
-      <x:c r="I11" s="41" t="e">
-        <x:f>HYPERLINK("https://www.noon.com/egypt-en/f2069-rgb-light-10-clock-mode-cooling-pad-cool-for-laptop-low-noise-fan-cooler-with-cell-phone-holder/N70023962V/p/","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.noon.com/egypt-en/f2069-rgb-light-10-clock-mode-cooling-pad-cool-for-laptop-low-noise-fan-cooler-with-cell-phone-holder/N70023962V/p/, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I11" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J11" s="26" t="str">
         <x:v>https://www.noon.com/egypt-en/f2069-rgb-light-10-clock-mode-cooling-pad-cool-for-laptop-low-noise-fan-cooler-with-cell-phone-holder/N70023962V/p/</x:v>
       </x:c>
-      <x:c r="K11" s="41" t="e">
-        <x:f>HYPERLINK("https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K11" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L11" s="26" t="str">
         <x:v>https://www.prohavit.com/zh-hans-jp/products/hv-f2069-laptop-cooling-pad-for-up-to-17-inch-laptop</x:v>
@@ -3045,16 +3033,14 @@
       <x:c r="H12" s="26" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="I12" s="41" t="e">
-        <x:f>HYPERLINK("https://www.amazon.eg/-/en/dp/B0DJH1W2N4","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.amazon.eg/-/en/dp/B0DJH1W2N4, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I12" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J12" s="26" t="str">
         <x:v>https://www.amazon.eg/-/en/dp/B0DJH1W2N4</x:v>
       </x:c>
-      <x:c r="K12" s="41" t="e">
-        <x:f>HYPERLINK("https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K12" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L12" s="26" t="str">
         <x:v>https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c</x:v>
@@ -3085,16 +3071,14 @@
       <x:c r="H13" s="26" t="str">
         <x:v>Unverified — public terms do not establish Egypt eligibility</x:v>
       </x:c>
-      <x:c r="I13" s="41" t="e">
-        <x:f>HYPERLINK("https://www.noon.com/egypt-en/joyroom-cable-organiser-jr-zs368-magnetic-black-6-pcs/ZDB64AB2F8DE78C016649Z/p/?o=zdb64ab2f8de78c016649z-1","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.noon.com/egypt-en/joyroom-cable-organiser-jr-zs368-magnetic-black-6-pcs/ZDB64AB2F8DE78C016649Z/p/?o=zdb64ab2f8de78c016649z-1, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I13" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J13" s="26" t="str">
         <x:v>https://www.noon.com/egypt-en/joyroom-cable-organiser-jr-zs368-magnetic-black-6-pcs/ZDB64AB2F8DE78C016649Z/p/?o=zdb64ab2f8de78c016649z-1</x:v>
       </x:c>
-      <x:c r="K13" s="41" t="e">
-        <x:f>HYPERLINK("https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K13" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L13" s="26" t="str">
         <x:v>https://www.joyroom.com/products/joyroom-jr-zs368-magnetic-cable-organizer-9pcs-b2c</x:v>
@@ -3125,16 +3109,14 @@
       <x:c r="H14" s="26" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="I14" s="41" t="e">
-        <x:f>HYPERLINK("https://www.amazon.eg/-/en/dp/B09QWY7JYK","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.amazon.eg/-/en/dp/B09QWY7JYK, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I14" s="41" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J14" s="26" t="str">
         <x:v>https://www.amazon.eg/-/en/dp/B09QWY7JYK</x:v>
       </x:c>
-      <x:c r="K14" s="41" t="e">
-        <x:f>HYPERLINK("https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K14" s="41" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L14" s="26" t="str">
         <x:v>https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html</x:v>
@@ -3165,16 +3147,14 @@
       <x:c r="H15" s="27" t="str">
         <x:v>Unverified — public terms do not establish Egypt eligibility</x:v>
       </x:c>
-      <x:c r="I15" s="42" t="e">
-        <x:f>HYPERLINK("https://www.noon.com/egypt-en/signature-m650-wireless-mouse-for-small-to-medium-sized-hands-silent-clicks-5-buttons-bluetooth-multi-device-compatibility-400-dpi-nominal-value-10m-range-black/N53285882A/p/","OPEN EXACT LISTING")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.noon.com/egypt-en/signature-m650-wireless-mouse-for-small-to-medium-sized-hands-silent-clicks-5-buttons-bluetooth-multi-device-compatibility-400-dpi-nominal-value-10m-range-black/N53285882A/p/, friendlyName=OPEN EXACT LISTING</x:v>
+      <x:c r="I15" s="42" t="str">
+        <x:v>OPEN EXACT LISTING</x:v>
       </x:c>
       <x:c r="J15" s="27" t="str">
         <x:v>https://www.noon.com/egypt-en/signature-m650-wireless-mouse-for-small-to-medium-sized-hands-silent-clicks-5-buttons-bluetooth-multi-device-compatibility-400-dpi-nominal-value-10m-range-black/N53285882A/p/</x:v>
       </x:c>
-      <x:c r="K15" s="42" t="e">
-        <x:f>HYPERLINK("https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html","OPEN MANUFACTURER SOURCE")</x:f>
-        <x:v>HYPERLINK is not implemented. linkLocation=https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html, friendlyName=OPEN MANUFACTURER SOURCE</x:v>
+      <x:c r="K15" s="42" t="str">
+        <x:v>OPEN MANUFACTURER SOURCE</x:v>
       </x:c>
       <x:c r="L15" s="27" t="str">
         <x:v>https://www.logitech.com/en-us/products/mice/m650-signature-wireless-mouse.html</x:v>
@@ -3191,15 +3171,37 @@
   <x:conditionalFormatting sqref="H6:H15">
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Unverified"/>
   </x:conditionalFormatting>
+  <x:hyperlinks>
+    <x:hyperlink ref="I6" r:id="rId1" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K6" r:id="rId2" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I7" r:id="rId3" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K7" r:id="rId4" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I8" r:id="rId5" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K8" r:id="rId6" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I9" r:id="rId7" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K9" r:id="rId8" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I10" r:id="rId9" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K10" r:id="rId10" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I11" r:id="rId11" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K11" r:id="rId12" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I12" r:id="rId13" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K12" r:id="rId14" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I13" r:id="rId15" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K13" r:id="rId16" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I14" r:id="rId17" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K14" r:id="rId18" display="OPEN MANUFACTURER SOURCE"/>
+    <x:hyperlink ref="I15" r:id="rId19" display="OPEN EXACT LISTING"/>
+    <x:hyperlink ref="K15" r:id="rId20" display="OPEN MANUFACTURER SOURCE"/>
+  </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re66e98c12f734d15"/>
+    <x:tablePart r:id="R33e59fc262bf4df9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
@@ -3264,46 +3266,46 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="L2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="M2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
       <x:c r="N2" s="7" t="str">
-        <x:v>Egypt-locale qualitative search-language evidence. Autocomplete presence is not search volume, difficulty, market share, or a trend-rate claim.</x:v>
+        <x:v>Egypt-locale qualitative search-language evidence. No volume/trend-direction/growth dataset was available, so the five products are not trend-validated winners.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="9" customHeight="1"/>
@@ -5474,13 +5476,13 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf04fecdbc5cb4111"/>
+    <x:tablePart r:id="R747a9733004d4a4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
@@ -10131,13 +10133,13 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd808c720f304445b"/>
+    <x:tablePart r:id="R97b1c809f6894fe9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
@@ -10539,13 +10541,13 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0f5d3fa6d584fb6"/>
+    <x:tablePart r:id="Rbab2f3775d2d48a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
@@ -10965,7 +10967,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re6977f1e44564994"/>
+    <x:tablePart r:id="R1d9375e419414719"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>